<commit_message>
Add LDAP authentication, CSRF protection, and related WFM Watch operational features.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Watcher_Analysis.xlsx
+++ b/docs/Watcher_Analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zebra-my.sharepoint.com/personal/sm5587_zebra_com/Documents/Daily_Work/WFMControlM/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="8_{E6A7E020-26C9-4B36-A237-A0D0F7FFF005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{749990D6-C27F-4B2D-AE3E-9623B8F7F9FE}"/>
+  <xr:revisionPtr revIDLastSave="174" documentId="8_{E6A7E020-26C9-4B36-A237-A0D0F7FFF005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCF190BF-F28D-4DDE-A544-44A05087ADE8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="115">
   <si>
     <t>Item #</t>
   </si>
@@ -317,6 +317,227 @@
     <t>Since WFM Watch is strictly an internal operations dashboard for global staff, the lack of per-client tenant isolation is an acceptable</t>
   </si>
   <si>
+    <t>JWT required on handshake; origins allowlisted; streams restricted by user permissions.</t>
+  </si>
+  <si>
+    <t>JWT denylist + tokenVersion invalidation; logout and admin revoke take effect immediately.</t>
+  </si>
+  <si>
+    <t>POST /api/auth/login is rate-limited to 10 failed login attempts per IP per 15 minutes; excess attempts receive HTTP 429.</t>
+  </si>
+  <si>
+    <t>DB polling intervals cannot be set below 5 minutes, and DB2 concurrency/pool settings are capped at 1–10; out-of-range values are rejected on config save.</t>
+  </si>
+  <si>
+    <t>Response on queries</t>
+  </si>
+  <si>
+    <t>Response on risks</t>
+  </si>
+  <si>
+    <r>
+      <t>Global Winston </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3B3B3B"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>redactFormat on all transports (JWTs, Bearer tokens, JDBC creds, sensitive JSON keys); remote log-tail API scrubbed via scrubRemoteLogLines(); Admin UI masks secrets.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>No automated procedure existed to rotate CONFIG_ENCRYPTION_KEY without outage. Resolution: Implemented dual-key rotation. During rotation, both keys are set in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0451A5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.env</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; decrypt tries the current key, then the previous key, so DB connections stay up. Admin runs Re-encrypt Secrets (pre-flight, then execute). After all secrets use the new key, remove </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3B3B3B"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CONFIG_ENCRYPTION_KEY_PREVIOUS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> and restart. The master key is never stored in the database.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Partially mitigated. DB2 passwords are decrypted only for short-lived </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Java 17 JDBC connector runs; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3B3B3B"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DB2_PASS_OVERRIDE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> is cleared from the child env after each exit; crypto Buffers are zero-filled. Full V8 heap scrubbing of JS strings is not possible in Node.js.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Client DB2 servers on port 50030 do not support TLS—JDBC with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3B3B3B"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>sslConnection=true</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> fails/times out, while plain JDBC succeeds—so application-level DB2 encryption cannot be enforced until DBA enables server-side DB2 SSL. Mitigated by deploying the app in a private subnet with egress firewall allowlists to registered client IPs only (ports 22, 50030, 587); DB2 credentials remain AES-256-GCM encrypted at rest. For SMTP, production enforces TLS via AppConfig (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3B3B3B"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>secrets.smtpTlsEnabled=true</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, port 587/465, certificate validation); local Mailpit dev is exempt. Operator access is protected by HTTPS at the nginx/load balancer with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3B3B3B"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>infra.trustProxy=true</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3B3B3B"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>infra.requireHttps=true</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Status:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> Partially mitigated—SMTP and app HTTPS are configurable at go-live; full DB2 transport encryption depends on DBA/infrastructure enabling DB2 TLS.</t>
+    </r>
+  </si>
+  <si>
+    <t>LDAP integration in progress.</t>
+  </si>
+  <si>
     <r>
       <t>WFM Watch now validates every cron log path before it is stored or passed to SSH. Paths must be absolute, stay under the configured WFM prefix (</t>
     </r>
@@ -328,12 +549,27 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>infra.sshWfmPathPrefix, default /mount/RWS4/) or /mount/backup, end in .log/.txt/.out, and must not contain .. or shell metacharacters. Invalid paths are dropped at job sync (with a server log warning) and are blocked again at log-check time and on the operator log-tail API (HTTP 400). Remote stat/tail commands use POSIX-safe quoting via a shared shellQuote() helper</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Client DB2 servers on port 50030 do not support TLS—JDBC with </t>
+      <t>infra.sshWfmPathPrefix, default /mount/RWS4/) or /mount/backup, end in .log/.txt/.out, and must not contain .. or shell metacharacters. Invalid paths are dropped at job sync (with a server log warning) and are blocked again at log-check time and on the operator log-tail API (HTTP 400). Remote stat/tail commands use POSIX-safe quoting via a shared shellQuote() helper.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Session JWT stored in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>HttpOnly, SameSite=Strict cookie; token inaccessible to JavaScript.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>JWTs use HS256 with an explicit verification allowlist (</t>
     </r>
     <r>
       <rPr>
@@ -343,12 +579,36 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>sslConnection=true fails/timeouts, while plain JDBC succeeds—so application-level DB2 encryption cannot be enforced until DBA enables server-side DB2 SSL; this is mitigated by deploying the app in a private subnet with egress firewall allowlists to registered client IPs only (ports 22, 50030, 587), and DB2 credentials remain AES-256-GCM encrypted at rest. For SMTP, production will enforce TLS via AppConfig (secrets.smtpTlsEnabled=true, port 587/465, certificate validation); local Mailpit dev is exempt. Operator access is protected by HTTPS at the nginx/load balancer with infra.trustProxy=true and infra.requireHttps=true. Status: Partially mitigated—SMTP and app HTTPS are configurable at go-live; full DB2 transport encryption depends on DBA/infrastructure enabling DB2 TLS.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Partially mitigated (Aug 2026). DB2 passwords are decrypted only for short-lived </t>
+      <t>algorithms: ['HS256']</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>), blocking none-algorithm and algorithm-switching attacks.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>WFM Watch enforces a read-only SSH command allowlist and path validation before every remote exec(app side)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Removed deprecated Nashorn/Java 8 bridge; DB2 access uses compiled </t>
     </r>
     <r>
       <rPr>
@@ -358,85 +618,18 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>jjs connector runs; DB2_PASS_OVERRIDE is cleared from the child env after each exit; crypto Buffers are zero-filled; Keeper passwords are no longer cached. Full V8 heap scrubbing of JS strings is not possible in Node.js.</t>
-    </r>
-  </si>
-  <si>
-    <t>Removed deprecated Nashorn/Java 8 DB2 bridge (→ Java 17 JDBC); minimized password lifetime in memory; DB2/SMTP/app HTTPS documented with compensating controls where server-side TLS is unavailable.</t>
-  </si>
-  <si>
-    <t>JWT required on handshake; origins allowlisted; streams restricted by user permissions.</t>
-  </si>
-  <si>
-    <t>all application logs pass through a redaction filter; log-tail responses are scrubbed.</t>
-  </si>
-  <si>
-    <r>
-      <t>No automated procedure to rotate </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF3B3B3B"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>CONFIG_ENCRYPTION_KEY</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t> without outage.  Resolution: Implemented dual-key rotation. During rotation, both keys are in .env; decrypt tries current then previous so DB connections stay up. Admin runs Re-encrypt Secrets (pre-flight → execute). After all secrets use the new key, remove _PREVIOUS and restart. Master key is never stored in the database.</t>
-    </r>
-  </si>
-  <si>
-    <t>JWT denylist + tokenVersion invalidation; logout and admin revoke take effect immediately.</t>
-  </si>
-  <si>
-    <t>HttpOnly cookie; token inaccessible to JavaScript.</t>
-  </si>
-  <si>
-    <r>
-      <t>JWTs use </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF3B3B3B"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>HS256 with an explicit verification allowlist (algorithms: ['HS256']), blocking none-algorithm and algorithm-switching attacks; </t>
-    </r>
-  </si>
-  <si>
-    <t>WFM Watch enforces a read-only SSH command allowlist and path validation before every remote exec.</t>
-  </si>
-  <si>
-    <t>POST /api/auth/login is rate-limited to 10 failed login attempts per IP per 15 minutes; excess attempts receive HTTP 429.</t>
-  </si>
-  <si>
-    <t>DB polling intervals cannot be set below 5 minutes, and DB2 concurrency/pool settings are capped at 1–10; out-of-range values are rejected on config save.</t>
-  </si>
-  <si>
-    <t>Response on queries</t>
-  </si>
-  <si>
-    <t>Response on risks</t>
+      <t>Java 17 JDBC connector; OpenJDK 17 in prod Docker. Optional future: native Node ibm_db driver.</t>
+    </r>
+  </si>
+  <si>
+    <t>Working with Infra team on the approach to be taken.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -469,6 +662,26 @@
       <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0451A5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -518,7 +731,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -532,7 +745,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -540,6 +753,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -853,12 +1069,13 @@
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.44140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="49.88671875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="51.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="43.109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="45.109375" style="2" customWidth="1"/>
     <col min="4" max="4" width="27.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.77734375" style="8" customWidth="1"/>
+    <col min="5" max="5" width="33.77734375" style="8" customWidth="1"/>
     <col min="6" max="6" width="66.21875" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="8.77734375" style="2"/>
+    <col min="7" max="7" width="34.109375" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="8.77734375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -869,7 +1086,7 @@
         <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
@@ -878,10 +1095,10 @@
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="144" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -899,7 +1116,7 @@
       </c>
       <c r="F2" s="6"/>
     </row>
-    <row r="3" spans="1:8" ht="144" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -915,11 +1132,12 @@
       <c r="E3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="F3" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="G3" s="4"/>
+    </row>
+    <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -935,12 +1153,13 @@
       <c r="E4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>100</v>
-      </c>
+      <c r="F4" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="G4" s="4"/>
       <c r="H4" s="5"/>
     </row>
-    <row r="5" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -992,11 +1211,11 @@
       <c r="E7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="F7" s="9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1011,6 +1230,9 @@
       </c>
       <c r="E8" s="8" t="s">
         <v>22</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -1030,7 +1252,7 @@
         <v>25</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
@@ -1086,7 +1308,7 @@
         <v>33</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
@@ -1142,7 +1364,7 @@
         <v>42</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -1161,11 +1383,11 @@
       <c r="E16" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="F16" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1182,10 +1404,11 @@
         <v>48</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+        <v>111</v>
+      </c>
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1202,10 +1425,10 @@
         <v>51</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1223,7 +1446,7 @@
       </c>
       <c r="F19" s="6"/>
     </row>
-    <row r="20" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1240,10 +1463,10 @@
         <v>57</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1261,7 +1484,7 @@
       </c>
       <c r="F21" s="6"/>
     </row>
-    <row r="22" spans="1:6" ht="144" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" ht="144" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1279,7 +1502,7 @@
       </c>
       <c r="F22" s="6"/>
     </row>
-    <row r="23" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1295,8 +1518,11 @@
       <c r="E23" s="8" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="F23" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1314,7 +1540,7 @@
       </c>
       <c r="F24" s="6"/>
     </row>
-    <row r="25" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1330,11 +1556,11 @@
       <c r="E25" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="F25" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1352,7 +1578,7 @@
       </c>
       <c r="F26" s="6"/>
     </row>
-    <row r="27" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1369,10 +1595,10 @@
         <v>78</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1390,7 +1616,7 @@
       </c>
       <c r="F28" s="6"/>
     </row>
-    <row r="29" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1406,8 +1632,8 @@
       <c r="E29" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="F29" s="2" t="s">
-        <v>101</v>
+      <c r="F29" s="4" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>